<commit_message>
chore: refresh LP pair rankings workbook
</commit_message>
<xml_diff>
--- a/LP-Pair-Rankings.xlsx
+++ b/LP-Pair-Rankings.xlsx
@@ -1011,7 +1011,7 @@
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U5" s="6" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="T7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U7" s="6" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="T9" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U9" s="6" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="T10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U10" s="6" t="inlineStr">
@@ -1527,7 +1527,7 @@
       </c>
       <c r="T11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U11" s="6" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="T12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U12" s="6" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="T13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U13" s="6" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="T14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U14" s="6" t="inlineStr">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="T15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U15" s="6" t="inlineStr">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="T16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U16" s="6" t="inlineStr">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="T17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U17" s="6" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="T18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U18" s="6" t="inlineStr">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="T19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U19" s="6" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U20" s="6" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="T21" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U21" s="6" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="T22" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U22" s="6" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U23" s="6" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="T24" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U24" s="6" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="T25" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U25" s="6" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="T26" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U26" s="6" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="T27" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U27" s="6" t="inlineStr">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="T28" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U28" s="6" t="inlineStr">
@@ -3079,7 +3079,7 @@
       </c>
       <c r="T29" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U29" s="6" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="T30" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U30" s="6" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="T31" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U31" s="6" t="inlineStr">
@@ -3337,7 +3337,7 @@
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U32" s="6" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="T33" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U33" s="6" t="inlineStr">
@@ -3509,7 +3509,7 @@
       </c>
       <c r="T34" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U34" s="6" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="T35" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U35" s="6" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="T36" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U36" s="6" t="inlineStr">
@@ -3767,7 +3767,7 @@
       </c>
       <c r="T37" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U37" s="6" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="T38" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U38" s="6" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="T39" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U39" s="6" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="T40" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U40" s="6" t="inlineStr">
@@ -4111,7 +4111,7 @@
       </c>
       <c r="T41" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U41" s="6" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="T42" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U42" s="6" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="T43" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U43" s="6" t="inlineStr">
@@ -4373,7 +4373,7 @@
       </c>
       <c r="T44" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U44" s="6" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="T45" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U45" s="6" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="T46" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U46" s="6" t="inlineStr">
@@ -4631,7 +4631,7 @@
       </c>
       <c r="T47" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U47" s="6" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U5" s="6" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="T7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U7" s="6" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U5" s="6" t="inlineStr">
@@ -5515,7 +5515,7 @@
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
@@ -5601,7 +5601,7 @@
       </c>
       <c r="T7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U7" s="6" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
@@ -5773,7 +5773,7 @@
       </c>
       <c r="T9" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U9" s="6" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="T10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U10" s="6" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="T11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U11" s="6" t="inlineStr">
@@ -6215,7 +6215,7 @@
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U5" s="6" t="inlineStr">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="T7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U7" s="6" t="inlineStr">
@@ -6485,7 +6485,7 @@
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
@@ -6759,7 +6759,7 @@
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U5" s="6" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="T6" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U6" s="6" t="inlineStr">
@@ -6931,7 +6931,7 @@
       </c>
       <c r="T7" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U7" s="6" t="inlineStr">
@@ -7017,7 +7017,7 @@
       </c>
       <c r="T8" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U8" s="6" t="inlineStr">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="T9" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U9" s="6" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="T10" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U10" s="6" t="inlineStr">
@@ -7275,7 +7275,7 @@
       </c>
       <c r="T11" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U11" s="6" t="inlineStr">
@@ -7361,7 +7361,7 @@
       </c>
       <c r="T12" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U12" s="6" t="inlineStr">
@@ -7447,7 +7447,7 @@
       </c>
       <c r="T13" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U13" s="6" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="T14" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U14" s="6" t="inlineStr">
@@ -7619,7 +7619,7 @@
       </c>
       <c r="T15" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U15" s="6" t="inlineStr">
@@ -7705,7 +7705,7 @@
       </c>
       <c r="T16" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U16" s="6" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="T17" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U17" s="6" t="inlineStr">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="T18" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U18" s="6" t="inlineStr">
@@ -7963,7 +7963,7 @@
       </c>
       <c r="T19" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U19" s="6" t="inlineStr">
@@ -8049,7 +8049,7 @@
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U20" s="6" t="inlineStr">
@@ -8135,7 +8135,7 @@
       </c>
       <c r="T21" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U21" s="6" t="inlineStr">
@@ -8221,7 +8221,7 @@
       </c>
       <c r="T22" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U22" s="6" t="inlineStr">
@@ -8307,7 +8307,7 @@
       </c>
       <c r="T23" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U23" s="6" t="inlineStr">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="T24" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U24" s="6" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="T25" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U25" s="6" t="inlineStr">
@@ -8565,7 +8565,7 @@
       </c>
       <c r="T26" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U26" s="6" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="T27" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U27" s="6" t="inlineStr">
@@ -8737,7 +8737,7 @@
       </c>
       <c r="T28" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U28" s="6" t="inlineStr">
@@ -8823,7 +8823,7 @@
       </c>
       <c r="T29" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U29" s="6" t="inlineStr">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="T30" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U30" s="6" t="inlineStr">
@@ -8995,7 +8995,7 @@
       </c>
       <c r="T31" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U31" s="6" t="inlineStr">
@@ -9081,7 +9081,7 @@
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U32" s="6" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="T33" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U33" s="6" t="inlineStr">
@@ -9253,7 +9253,7 @@
       </c>
       <c r="T34" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U34" s="6" t="inlineStr">
@@ -9339,7 +9339,7 @@
       </c>
       <c r="T35" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U35" s="6" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="T36" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U36" s="6" t="inlineStr">
@@ -9511,7 +9511,7 @@
       </c>
       <c r="T37" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U37" s="6" t="inlineStr">
@@ -9597,7 +9597,7 @@
       </c>
       <c r="T38" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U38" s="6" t="inlineStr">
@@ -9683,7 +9683,7 @@
       </c>
       <c r="T39" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U39" s="6" t="inlineStr">
@@ -9769,7 +9769,7 @@
       </c>
       <c r="T40" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U40" s="6" t="inlineStr">
@@ -9855,7 +9855,7 @@
       </c>
       <c r="T41" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U41" s="6" t="inlineStr">
@@ -9941,7 +9941,7 @@
       </c>
       <c r="T42" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U42" s="6" t="inlineStr">
@@ -10027,7 +10027,7 @@
       </c>
       <c r="T43" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U43" s="6" t="inlineStr">
@@ -10113,7 +10113,7 @@
       </c>
       <c r="T44" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U44" s="6" t="inlineStr">
@@ -10199,7 +10199,7 @@
       </c>
       <c r="T45" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U45" s="6" t="inlineStr">
@@ -10285,7 +10285,7 @@
       </c>
       <c r="T46" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U46" s="6" t="inlineStr">
@@ -10371,7 +10371,7 @@
       </c>
       <c r="T47" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U47" s="6" t="inlineStr">
@@ -10457,7 +10457,7 @@
       </c>
       <c r="T48" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U48" s="6" t="inlineStr">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="T49" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U49" s="6" t="inlineStr">
@@ -10629,7 +10629,7 @@
       </c>
       <c r="T50" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U50" s="6" t="inlineStr">
@@ -10715,7 +10715,7 @@
       </c>
       <c r="T51" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U51" s="6" t="inlineStr">
@@ -10801,7 +10801,7 @@
       </c>
       <c r="T52" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U52" s="6" t="inlineStr">
@@ -10887,7 +10887,7 @@
       </c>
       <c r="T53" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U53" s="6" t="inlineStr">
@@ -10973,7 +10973,7 @@
       </c>
       <c r="T54" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U54" s="6" t="inlineStr">
@@ -11059,7 +11059,7 @@
       </c>
       <c r="T55" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U55" s="6" t="inlineStr">
@@ -11145,7 +11145,7 @@
       </c>
       <c r="T56" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U56" s="6" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="T57" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U57" s="6" t="inlineStr">
@@ -11317,7 +11317,7 @@
       </c>
       <c r="T58" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U58" s="6" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="T59" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U59" s="6" t="inlineStr">
@@ -11489,7 +11489,7 @@
       </c>
       <c r="T60" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U60" s="6" t="inlineStr">
@@ -11579,7 +11579,7 @@
       </c>
       <c r="T61" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U61" s="6" t="inlineStr">
@@ -11665,7 +11665,7 @@
       </c>
       <c r="T62" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U62" s="6" t="inlineStr">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="T63" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U63" s="6" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="T64" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U64" s="6" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="T65" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U65" s="6" t="inlineStr">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="T66" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U66" s="6" t="inlineStr">
@@ -12095,7 +12095,7 @@
       </c>
       <c r="T67" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U67" s="6" t="inlineStr">
@@ -12181,7 +12181,7 @@
       </c>
       <c r="T68" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U68" s="6" t="inlineStr">
@@ -12267,7 +12267,7 @@
       </c>
       <c r="T69" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U69" s="6" t="inlineStr">
@@ -12353,7 +12353,7 @@
       </c>
       <c r="T70" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U70" s="6" t="inlineStr">
@@ -12439,7 +12439,7 @@
       </c>
       <c r="T71" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U71" s="6" t="inlineStr">
@@ -12525,7 +12525,7 @@
       </c>
       <c r="T72" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U72" s="6" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="T73" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U73" s="6" t="inlineStr">
@@ -12697,7 +12697,7 @@
       </c>
       <c r="T74" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U74" s="6" t="inlineStr">
@@ -12783,7 +12783,7 @@
       </c>
       <c r="T75" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U75" s="6" t="inlineStr">
@@ -12869,7 +12869,7 @@
       </c>
       <c r="T76" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U76" s="6" t="inlineStr">
@@ -12955,7 +12955,7 @@
       </c>
       <c r="T77" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U77" s="6" t="inlineStr">
@@ -13041,7 +13041,7 @@
       </c>
       <c r="T78" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U78" s="6" t="inlineStr">
@@ -13127,7 +13127,7 @@
       </c>
       <c r="T79" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U79" s="6" t="inlineStr">
@@ -13213,7 +13213,7 @@
       </c>
       <c r="T80" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U80" s="6" t="inlineStr">
@@ -13299,7 +13299,7 @@
       </c>
       <c r="T81" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U81" s="6" t="inlineStr">
@@ -13385,7 +13385,7 @@
       </c>
       <c r="T82" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U82" s="6" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="T83" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U83" s="6" t="inlineStr">
@@ -13557,7 +13557,7 @@
       </c>
       <c r="T84" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U84" s="6" t="inlineStr">
@@ -13643,7 +13643,7 @@
       </c>
       <c r="T85" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U85" s="6" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="T86" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U86" s="6" t="inlineStr">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="T87" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U87" s="6" t="inlineStr">
@@ -13901,7 +13901,7 @@
       </c>
       <c r="T88" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U88" s="6" t="inlineStr">
@@ -13987,7 +13987,7 @@
       </c>
       <c r="T89" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U89" s="6" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="T90" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U90" s="6" t="inlineStr">
@@ -14159,7 +14159,7 @@
       </c>
       <c r="T91" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U91" s="6" t="inlineStr">
@@ -14245,7 +14245,7 @@
       </c>
       <c r="T92" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U92" s="6" t="inlineStr">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="T93" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U93" s="6" t="inlineStr">
@@ -14417,7 +14417,7 @@
       </c>
       <c r="T94" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U94" s="6" t="inlineStr">
@@ -14503,7 +14503,7 @@
       </c>
       <c r="T95" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U95" s="6" t="inlineStr">
@@ -14589,7 +14589,7 @@
       </c>
       <c r="T96" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U96" s="6" t="inlineStr">
@@ -14675,7 +14675,7 @@
       </c>
       <c r="T97" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U97" s="6" t="inlineStr">
@@ -14761,7 +14761,7 @@
       </c>
       <c r="T98" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U98" s="6" t="inlineStr">
@@ -14847,7 +14847,7 @@
       </c>
       <c r="T99" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U99" s="6" t="inlineStr">
@@ -14933,7 +14933,7 @@
       </c>
       <c r="T100" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U100" s="6" t="inlineStr">
@@ -15019,7 +15019,7 @@
       </c>
       <c r="T101" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U101" s="6" t="inlineStr">
@@ -15105,7 +15105,7 @@
       </c>
       <c r="T102" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U102" s="6" t="inlineStr">
@@ -15191,7 +15191,7 @@
       </c>
       <c r="T103" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U103" s="6" t="inlineStr">
@@ -15277,7 +15277,7 @@
       </c>
       <c r="T104" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U104" s="6" t="inlineStr">
@@ -15363,7 +15363,7 @@
       </c>
       <c r="T105" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U105" s="6" t="inlineStr">
@@ -15449,7 +15449,7 @@
       </c>
       <c r="T106" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U106" s="6" t="inlineStr">
@@ -15535,7 +15535,7 @@
       </c>
       <c r="T107" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U107" s="6" t="inlineStr">
@@ -15621,7 +15621,7 @@
       </c>
       <c r="T108" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U108" s="6" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="T109" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U109" s="6" t="inlineStr">
@@ -15793,7 +15793,7 @@
       </c>
       <c r="T110" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U110" s="6" t="inlineStr">
@@ -15879,7 +15879,7 @@
       </c>
       <c r="T111" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U111" s="6" t="inlineStr">
@@ -15965,7 +15965,7 @@
       </c>
       <c r="T112" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U112" s="6" t="inlineStr">
@@ -16051,7 +16051,7 @@
       </c>
       <c r="T113" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U113" s="6" t="inlineStr">
@@ -16137,7 +16137,7 @@
       </c>
       <c r="T114" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U114" s="6" t="inlineStr">
@@ -16223,7 +16223,7 @@
       </c>
       <c r="T115" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U115" s="6" t="inlineStr">
@@ -16309,7 +16309,7 @@
       </c>
       <c r="T116" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U116" s="6" t="inlineStr">
@@ -16395,7 +16395,7 @@
       </c>
       <c r="T117" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U117" s="6" t="inlineStr">
@@ -16481,7 +16481,7 @@
       </c>
       <c r="T118" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U118" s="6" t="inlineStr">
@@ -16567,7 +16567,7 @@
       </c>
       <c r="T119" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U119" s="6" t="inlineStr">
@@ -16653,7 +16653,7 @@
       </c>
       <c r="T120" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U120" s="6" t="inlineStr">
@@ -16739,7 +16739,7 @@
       </c>
       <c r="T121" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U121" s="6" t="inlineStr">
@@ -16825,7 +16825,7 @@
       </c>
       <c r="T122" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U122" s="6" t="inlineStr">
@@ -16911,7 +16911,7 @@
       </c>
       <c r="T123" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U123" s="6" t="inlineStr">
@@ -16997,7 +16997,7 @@
       </c>
       <c r="T124" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U124" s="6" t="inlineStr">
@@ -17083,7 +17083,7 @@
       </c>
       <c r="T125" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U125" s="6" t="inlineStr">
@@ -17169,7 +17169,7 @@
       </c>
       <c r="T126" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U126" s="6" t="inlineStr">
@@ -17255,7 +17255,7 @@
       </c>
       <c r="T127" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U127" s="6" t="inlineStr">
@@ -17341,7 +17341,7 @@
       </c>
       <c r="T128" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U128" s="6" t="inlineStr">
@@ -17427,7 +17427,7 @@
       </c>
       <c r="T129" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U129" s="6" t="inlineStr">
@@ -17513,7 +17513,7 @@
       </c>
       <c r="T130" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U130" s="6" t="inlineStr">
@@ -17599,7 +17599,7 @@
       </c>
       <c r="T131" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U131" s="6" t="inlineStr">
@@ -17685,7 +17685,7 @@
       </c>
       <c r="T132" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U132" s="6" t="inlineStr">
@@ -17775,7 +17775,7 @@
       </c>
       <c r="T133" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U133" s="6" t="inlineStr">
@@ -17861,7 +17861,7 @@
       </c>
       <c r="T134" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U134" s="6" t="inlineStr">
@@ -17947,7 +17947,7 @@
       </c>
       <c r="T135" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U135" s="6" t="inlineStr">
@@ -18033,7 +18033,7 @@
       </c>
       <c r="T136" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U136" s="6" t="inlineStr">
@@ -18123,7 +18123,7 @@
       </c>
       <c r="T137" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U137" s="6" t="inlineStr">
@@ -18209,7 +18209,7 @@
       </c>
       <c r="T138" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U138" s="6" t="inlineStr">
@@ -18295,7 +18295,7 @@
       </c>
       <c r="T139" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U139" s="6" t="inlineStr">
@@ -18381,7 +18381,7 @@
       </c>
       <c r="T140" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U140" s="6" t="inlineStr">
@@ -18467,7 +18467,7 @@
       </c>
       <c r="T141" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U141" s="6" t="inlineStr">
@@ -18553,7 +18553,7 @@
       </c>
       <c r="T142" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U142" s="6" t="inlineStr">
@@ -18639,7 +18639,7 @@
       </c>
       <c r="T143" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U143" s="6" t="inlineStr">
@@ -18725,7 +18725,7 @@
       </c>
       <c r="T144" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U144" s="6" t="inlineStr">
@@ -18811,7 +18811,7 @@
       </c>
       <c r="T145" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U145" s="6" t="inlineStr">
@@ -18897,7 +18897,7 @@
       </c>
       <c r="T146" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U146" s="6" t="inlineStr">
@@ -18983,7 +18983,7 @@
       </c>
       <c r="T147" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U147" s="6" t="inlineStr">
@@ -19069,7 +19069,7 @@
       </c>
       <c r="T148" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U148" s="6" t="inlineStr">
@@ -19155,7 +19155,7 @@
       </c>
       <c r="T149" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U149" s="6" t="inlineStr">
@@ -19241,7 +19241,7 @@
       </c>
       <c r="T150" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U150" s="6" t="inlineStr">
@@ -19327,7 +19327,7 @@
       </c>
       <c r="T151" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U151" s="6" t="inlineStr">
@@ -19413,7 +19413,7 @@
       </c>
       <c r="T152" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U152" s="6" t="inlineStr">
@@ -19499,7 +19499,7 @@
       </c>
       <c r="T153" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U153" s="6" t="inlineStr">
@@ -19585,7 +19585,7 @@
       </c>
       <c r="T154" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U154" s="6" t="inlineStr">
@@ -19671,7 +19671,7 @@
       </c>
       <c r="T155" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U155" s="6" t="inlineStr">
@@ -19757,7 +19757,7 @@
       </c>
       <c r="T156" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U156" s="6" t="inlineStr">
@@ -19843,7 +19843,7 @@
       </c>
       <c r="T157" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U157" s="6" t="inlineStr">
@@ -19929,7 +19929,7 @@
       </c>
       <c r="T158" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U158" s="6" t="inlineStr">
@@ -20015,7 +20015,7 @@
       </c>
       <c r="T159" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U159" s="6" t="inlineStr">
@@ -20101,7 +20101,7 @@
       </c>
       <c r="T160" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U160" s="6" t="inlineStr">
@@ -20187,7 +20187,7 @@
       </c>
       <c r="T161" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U161" s="6" t="inlineStr">
@@ -20273,7 +20273,7 @@
       </c>
       <c r="T162" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U162" s="6" t="inlineStr">
@@ -20359,7 +20359,7 @@
       </c>
       <c r="T163" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U163" s="6" t="inlineStr">
@@ -20445,7 +20445,7 @@
       </c>
       <c r="T164" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U164" s="6" t="inlineStr">
@@ -20535,7 +20535,7 @@
       </c>
       <c r="T165" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U165" s="6" t="inlineStr">
@@ -20621,7 +20621,7 @@
       </c>
       <c r="T166" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U166" s="6" t="inlineStr">
@@ -20707,7 +20707,7 @@
       </c>
       <c r="T167" s="6" t="inlineStr">
         <is>
-          <t>2026-09-25T15:22:42+00:00</t>
+          <t>2026-09-25T15:23:08+00:00</t>
         </is>
       </c>
       <c r="U167" s="6" t="inlineStr">

</xml_diff>